<commit_message>
For Screenshot.xlsx: Assumptions, Revenue Build and Cost Build behind Profit and Loss
Formulas across sheets for Trace Tree screenshots: net profit traces back 13 levels through five sheets.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/For Screenshot.xlsx
+++ b/For Screenshot.xlsx
@@ -5,23 +5,26 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juihn\Source\Repos\tinykit-excel-releases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juihn\AppData\Local\Temp\claude\C--Users-juihn-Source-Repos\4da50449-f373-4d59-a192-72dd6ebbb527\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D91F3F3-D6E5-4370-A4B8-BF25B641976E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1DEBCC3-C6C7-4F33-9078-6AB1134CAF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Balance Sheet" sheetId="1" r:id="rId1"/>
     <sheet name="Cashflow Statement" sheetId="2" r:id="rId2"/>
     <sheet name="Profit and Loss" sheetId="3" r:id="rId3"/>
+    <sheet name="Revenue Build" sheetId="4" r:id="rId4"/>
+    <sheet name="Cost Build" sheetId="5" r:id="rId5"/>
+    <sheet name="Assumptions" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="ClosingCash">'Cashflow Statement'!$D$32:$F$32</definedName>
     <definedName name="NetProfit">'Profit and Loss'!$D$35:$F$35</definedName>
     <definedName name="Revenue">'Profit and Loss'!$D$10:$F$10</definedName>
-    <definedName name="TaxRate">'Profit and Loss'!$D$39</definedName>
+    <definedName name="TaxRate">Assumptions!$D$32</definedName>
     <definedName name="TotalAssets">'Balance Sheet'!$D$20:$F$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="127">
   <si>
     <t>Northwind Components Ltd. (fictional)</t>
   </si>
@@ -302,22 +305,137 @@
     <t>Net margin</t>
   </si>
   <si>
+    <t>Revenue Build</t>
+  </si>
+  <si>
+    <t>Product sales and services, from Assumptions ($ in thousands unless stated)</t>
+  </si>
+  <si>
+    <t>Widgets</t>
+  </si>
+  <si>
+    <t>Units sold</t>
+  </si>
+  <si>
+    <t>Price per widget ($)</t>
+  </si>
+  <si>
+    <t>Service contracts</t>
+  </si>
+  <si>
+    <t>Average fee per contract</t>
+  </si>
+  <si>
+    <t>Service revenue</t>
+  </si>
+  <si>
+    <t>Cost Build</t>
+  </si>
+  <si>
+    <t>Costs and interest, from Assumptions, Revenue Build and Balance Sheet ($ in thousands)</t>
+  </si>
+  <si>
+    <t>Material cost per widget ($)</t>
+  </si>
+  <si>
+    <t>Labour hours (thousands)</t>
+  </si>
+  <si>
+    <t>Salaries</t>
+  </si>
+  <si>
+    <t>Other operating expenses</t>
+  </si>
+  <si>
+    <t>Interest</t>
+  </si>
+  <si>
+    <t>Borrowings at year end</t>
+  </si>
+  <si>
     <t>Assumptions</t>
   </si>
   <si>
+    <t>Inputs behind Profit and Loss (all fictional)</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>Widgets sold, FY2023 (units)</t>
+  </si>
+  <si>
+    <t>Volume growth</t>
+  </si>
+  <si>
+    <t>Price per widget, FY2023 ($)</t>
+  </si>
+  <si>
+    <t>Price increase</t>
+  </si>
+  <si>
+    <t>Service contracts, FY2023</t>
+  </si>
+  <si>
+    <t>Contract growth</t>
+  </si>
+  <si>
+    <t>Average fee per contract ($000)</t>
+  </si>
+  <si>
+    <t>Costs</t>
+  </si>
+  <si>
+    <t>Material cost per widget, FY2023 ($)</t>
+  </si>
+  <si>
+    <t>Material cost inflation</t>
+  </si>
+  <si>
+    <t>Labour hours per widget</t>
+  </si>
+  <si>
+    <t>Labour rate ($ per hour)</t>
+  </si>
+  <si>
+    <t>People</t>
+  </si>
+  <si>
+    <t>Sales headcount</t>
+  </si>
+  <si>
+    <t>Administrative headcount</t>
+  </si>
+  <si>
+    <t>Average salary, sales ($000)</t>
+  </si>
+  <si>
+    <t>Average salary, administrative ($000)</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Advertising, % of total revenue</t>
+  </si>
+  <si>
+    <t>Office rent ($000)</t>
+  </si>
+  <si>
+    <t>Interest rate on borrowings</t>
+  </si>
+  <si>
     <t>Income tax rate</t>
-  </si>
-  <si>
-    <t>Input: a fictional rate for this example</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%;\(0.0%\);&quot;-&quot;"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -331,51 +449,43 @@
       <b/>
       <sz val="14"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF595959"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF008000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF808080"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -432,7 +542,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -441,15 +551,23 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,7 +602,6 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-GB"/>
               <a:t>Revenue and Net Profit ($ thousands)</a:t>
             </a:r>
           </a:p>
@@ -543,20 +660,20 @@
                 <c:formatCode>#,##0;\(#,##0\);"-"</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>48000</c:v>
+                  <c:v>47990</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>54000</c:v>
+                  <c:v>53957.377499999995</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>61000</c:v>
+                  <c:v>60757.229692500005</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5C5E-401E-85FB-152048C2EC90}"/>
+              <c16:uniqueId val="{00000000-DE1A-4CCB-9490-B96D56BABCDA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -601,20 +718,20 @@
                 <c:formatCode>#,##0;\(#,##0\);"-"</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>7882</c:v>
+                  <c:v>7946.99</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9637</c:v>
+                  <c:v>9342.0567474999916</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12097</c:v>
+                  <c:v>11393.025819582497</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-5C5E-401E-85FB-152048C2EC90}"/>
+              <c16:uniqueId val="{00000001-DE1A-4CCB-9490-B96D56BABCDA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -666,7 +783,6 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-GB"/>
                   <a:t>$ thousands</a:t>
                 </a:r>
               </a:p>
@@ -684,8 +800,8 @@
       </c:valAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
+      <c:legendPos val="r"/>
+      <c:overlay val="1"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
@@ -701,19 +817,14 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="4680000" cy="2700000"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -736,7 +847,7 @@
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1053,15 +1164,15 @@
       </c>
       <c r="D9" s="6">
         <f>'Cashflow Statement'!D32</f>
-        <v>8472</v>
+        <v>8536.99</v>
       </c>
       <c r="E9" s="6">
         <f>'Cashflow Statement'!E32</f>
-        <v>13759</v>
+        <v>13529.046747499991</v>
       </c>
       <c r="F9" s="6">
         <f>'Cashflow Statement'!F32</f>
-        <v>21426</v>
+        <v>20492.07256708249</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -1112,15 +1223,15 @@
       </c>
       <c r="D13" s="8">
         <f>SUM(D9:D12)</f>
-        <v>20102</v>
+        <v>20166.989999999998</v>
       </c>
       <c r="E13" s="8">
         <f>SUM(E9:E12)</f>
-        <v>26749</v>
+        <v>26519.04674749999</v>
       </c>
       <c r="F13" s="8">
         <f>SUM(F9:F12)</f>
-        <v>35676</v>
+        <v>34742.07256708249</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -1184,15 +1295,15 @@
       </c>
       <c r="D20" s="9">
         <f>D13+D18</f>
-        <v>37802</v>
+        <v>37866.99</v>
       </c>
       <c r="E20" s="9">
         <f>E13+E18</f>
-        <v>45269</v>
+        <v>45039.04674749999</v>
       </c>
       <c r="F20" s="9">
         <f>F13+F18</f>
-        <v>54696</v>
+        <v>53762.07256708249</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1341,15 +1452,15 @@
         <v>31</v>
       </c>
       <c r="D37" s="7">
-        <v>12172</v>
+        <v>12237</v>
       </c>
       <c r="E37" s="6">
         <f>D37+'Profit and Loss'!E35+'Cashflow Statement'!E27</f>
-        <v>20309</v>
+        <v>20079.056747499992</v>
       </c>
       <c r="F37" s="6">
         <f>E37+'Profit and Loss'!F35+'Cashflow Statement'!F27</f>
-        <v>30606</v>
+        <v>29672.082567082489</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>32</v>
@@ -1361,15 +1472,15 @@
       </c>
       <c r="D38" s="8">
         <f>SUM(D36:D37)</f>
-        <v>22172</v>
+        <v>22237</v>
       </c>
       <c r="E38" s="8">
         <f>SUM(E36:E37)</f>
-        <v>30309</v>
+        <v>30079.056747499992</v>
       </c>
       <c r="F38" s="8">
         <f>SUM(F36:F37)</f>
-        <v>40606</v>
+        <v>39672.082567082485</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
@@ -1378,15 +1489,15 @@
       </c>
       <c r="D40" s="10">
         <f>D33+D38</f>
-        <v>37802</v>
+        <v>37867</v>
       </c>
       <c r="E40" s="10">
         <f>E33+E38</f>
-        <v>45269</v>
+        <v>45039.056747499992</v>
       </c>
       <c r="F40" s="10">
         <f>F33+F38</f>
-        <v>54696</v>
+        <v>53762.082567082485</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
@@ -1458,15 +1569,15 @@
       </c>
       <c r="D8" s="6">
         <f>'Profit and Loss'!D35</f>
-        <v>7882</v>
+        <v>7946.99</v>
       </c>
       <c r="E8" s="6">
         <f>'Profit and Loss'!E35</f>
-        <v>9637</v>
+        <v>9342.0567474999916</v>
       </c>
       <c r="F8" s="6">
         <f>'Profit and Loss'!F35</f>
-        <v>12097</v>
+        <v>11393.025819582497</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -1580,15 +1691,15 @@
       </c>
       <c r="D16" s="8">
         <f>SUM(D8:D9)+SUM(D11:D15)</f>
-        <v>8972</v>
+        <v>9036.99</v>
       </c>
       <c r="E16" s="8">
         <f>SUM(E8:E9)+SUM(E11:E15)</f>
-        <v>10587</v>
+        <v>10292.056747499992</v>
       </c>
       <c r="F16" s="8">
         <f>SUM(F8:F9)+SUM(F11:F15)</f>
-        <v>13217</v>
+        <v>12513.025819582497</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -1733,15 +1844,15 @@
       </c>
       <c r="D30" s="9">
         <f>D16+D21+D28</f>
-        <v>5322</v>
+        <v>5386.99</v>
       </c>
       <c r="E30" s="9">
         <f>E16+E21+E28</f>
-        <v>5287</v>
+        <v>4992.0567474999916</v>
       </c>
       <c r="F30" s="9">
         <f>F16+F21+F28</f>
-        <v>7667</v>
+        <v>6963.0258195824972</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -1753,11 +1864,11 @@
       </c>
       <c r="E31" s="9">
         <f>D32</f>
-        <v>8472</v>
+        <v>8536.99</v>
       </c>
       <c r="F31" s="9">
         <f>E32</f>
-        <v>13759</v>
+        <v>13529.046747499991</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -1766,15 +1877,15 @@
       </c>
       <c r="D32" s="10">
         <f>D30+D31</f>
-        <v>8472</v>
+        <v>8536.99</v>
       </c>
       <c r="E32" s="10">
         <f>E30+E31</f>
-        <v>13759</v>
+        <v>13529.046747499991</v>
       </c>
       <c r="F32" s="10">
         <f>F30+F31</f>
-        <v>21426</v>
+        <v>20492.07256708249</v>
       </c>
     </row>
   </sheetData>
@@ -1784,12 +1895,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="3" customWidth="1"/>
-    <col min="3" max="3" width="22.5546875" customWidth="1"/>
-    <col min="4" max="6" width="6.88671875" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
@@ -1827,28 +1938,34 @@
       <c r="C8" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="7">
-        <v>38200</v>
-      </c>
-      <c r="E8" s="7">
-        <v>42650</v>
-      </c>
-      <c r="F8" s="7">
-        <v>47100</v>
+      <c r="D8" s="6">
+        <f>'Revenue Build'!D10</f>
+        <v>38190</v>
+      </c>
+      <c r="E8" s="6">
+        <f>'Revenue Build'!E10</f>
+        <v>42667.777499999997</v>
+      </c>
+      <c r="F8" s="6">
+        <f>'Revenue Build'!F10</f>
+        <v>47233.229692500005</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6">
+        <f>'Revenue Build'!D15</f>
         <v>9800</v>
       </c>
-      <c r="E9" s="7">
-        <v>11350</v>
-      </c>
-      <c r="F9" s="7">
-        <v>13900</v>
+      <c r="E9" s="6">
+        <f>'Revenue Build'!E15</f>
+        <v>11289.6</v>
+      </c>
+      <c r="F9" s="6">
+        <f>'Revenue Build'!F15</f>
+        <v>13524</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1857,15 +1974,15 @@
       </c>
       <c r="D10" s="8">
         <f>SUM(D8:D9)</f>
-        <v>48000</v>
+        <v>47990</v>
       </c>
       <c r="E10" s="8">
         <f>SUM(E8:E9)</f>
-        <v>54000</v>
+        <v>53957.377499999995</v>
       </c>
       <c r="F10" s="8">
         <f>SUM(F8:F9)</f>
-        <v>61000</v>
+        <v>60757.229692500005</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1877,28 +1994,34 @@
       <c r="C13" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="7">
-        <v>17190</v>
-      </c>
-      <c r="E13" s="7">
-        <v>18980</v>
-      </c>
-      <c r="F13" s="7">
-        <v>20720</v>
+      <c r="D13" s="6">
+        <f>'Cost Build'!D10</f>
+        <v>17195</v>
+      </c>
+      <c r="E13" s="6">
+        <f>'Cost Build'!E10</f>
+        <v>19304.826500000003</v>
+      </c>
+      <c r="F13" s="6">
+        <f>'Cost Build'!F10</f>
+        <v>21474.688998600006</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
         <v>69</v>
       </c>
-      <c r="D14" s="7">
-        <v>7640</v>
-      </c>
-      <c r="E14" s="7">
-        <v>8370</v>
-      </c>
-      <c r="F14" s="7">
-        <v>9310</v>
+      <c r="D14" s="6">
+        <f>'Cost Build'!D13</f>
+        <v>7600</v>
+      </c>
+      <c r="E14" s="6">
+        <f>'Cost Build'!E13</f>
+        <v>8507.6680000000015</v>
+      </c>
+      <c r="F14" s="6">
+        <f>'Cost Build'!F13</f>
+        <v>9420.8961600000021</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1907,15 +2030,15 @@
       </c>
       <c r="D15" s="8">
         <f>SUM(D13:D14)</f>
-        <v>24830</v>
+        <v>24795</v>
       </c>
       <c r="E15" s="8">
         <f>SUM(E13:E14)</f>
-        <v>27350</v>
+        <v>27812.494500000004</v>
       </c>
       <c r="F15" s="8">
         <f>SUM(F13:F14)</f>
-        <v>30030</v>
+        <v>30895.585158600006</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -1924,15 +2047,15 @@
       </c>
       <c r="D17" s="9">
         <f>D10-D15</f>
-        <v>23170</v>
+        <v>23195</v>
       </c>
       <c r="E17" s="9">
         <f>E10-E15</f>
-        <v>26650</v>
+        <v>26144.882999999991</v>
       </c>
       <c r="F17" s="9">
         <f>F10-F15</f>
-        <v>30970</v>
+        <v>29861.644533899998</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -1941,15 +2064,15 @@
       </c>
       <c r="D18" s="13">
         <f>IF(D10=0,0,D17/D10)</f>
-        <v>0.48270833333333335</v>
+        <v>0.48332986038758075</v>
       </c>
       <c r="E18" s="13">
         <f>IF(E10=0,0,E17/E10)</f>
-        <v>0.49351851851851852</v>
+        <v>0.48454695560398564</v>
       </c>
       <c r="F18" s="13">
         <f>IF(F10=0,0,F17/F10)</f>
-        <v>0.50770491803278683</v>
+        <v>0.49149121322735656</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -1966,28 +2089,34 @@
       <c r="C22" t="s">
         <v>75</v>
       </c>
-      <c r="D22" s="7">
-        <v>2350</v>
-      </c>
-      <c r="E22" s="7">
-        <v>2780</v>
-      </c>
-      <c r="F22" s="7">
-        <v>3120</v>
+      <c r="D22" s="6">
+        <f>'Cost Build'!D20</f>
+        <v>2351.5100000000002</v>
+      </c>
+      <c r="E22" s="6">
+        <f>'Cost Build'!E20</f>
+        <v>2751.8262524999996</v>
+      </c>
+      <c r="F22" s="6">
+        <f>'Cost Build'!F20</f>
+        <v>3098.6187143175002</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C23" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="6">
+        <f>'Cost Build'!D16</f>
         <v>3900</v>
       </c>
-      <c r="E23" s="7">
-        <v>4250</v>
-      </c>
-      <c r="F23" s="7">
-        <v>4600</v>
+      <c r="E23" s="6">
+        <f>'Cost Build'!E16</f>
+        <v>4262.5</v>
+      </c>
+      <c r="F23" s="6">
+        <f>'Cost Build'!F16</f>
+        <v>4582</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1999,13 +2128,16 @@
       <c r="C25" t="s">
         <v>78</v>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="6">
+        <f>'Cost Build'!D21</f>
         <v>1450</v>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="6">
+        <f>'Cost Build'!E21</f>
         <v>1500</v>
       </c>
-      <c r="F25" s="7">
+      <c r="F25" s="6">
+        <f>'Cost Build'!F21</f>
         <v>1560</v>
       </c>
     </row>
@@ -2013,14 +2145,17 @@
       <c r="C26" t="s">
         <v>79</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="6">
+        <f>'Cost Build'!D17</f>
         <v>2700</v>
       </c>
-      <c r="E26" s="7">
-        <v>2880</v>
-      </c>
-      <c r="F26" s="7">
-        <v>3050</v>
+      <c r="E26" s="6">
+        <f>'Cost Build'!E17</f>
+        <v>2883</v>
+      </c>
+      <c r="F26" s="6">
+        <f>'Cost Build'!F17</f>
+        <v>3040</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -2043,15 +2178,15 @@
       </c>
       <c r="D28" s="8">
         <f>SUM(D22:D23)+SUM(D25:D27)</f>
-        <v>12020</v>
+        <v>12021.51</v>
       </c>
       <c r="E28" s="8">
         <f>SUM(E22:E23)+SUM(E25:E27)</f>
-        <v>13190</v>
+        <v>13177.326252499999</v>
       </c>
       <c r="F28" s="8">
         <f>SUM(F22:F23)+SUM(F25:F27)</f>
-        <v>14280</v>
+        <v>14230.618714317501</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -2060,29 +2195,32 @@
       </c>
       <c r="D30" s="9">
         <f>D17-D28</f>
-        <v>11150</v>
+        <v>11173.49</v>
       </c>
       <c r="E30" s="9">
         <f>E17-E28</f>
-        <v>13460</v>
+        <v>12967.556747499992</v>
       </c>
       <c r="F30" s="9">
         <f>F17-F28</f>
-        <v>16690</v>
+        <v>15631.025819582497</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C31" t="s">
         <v>82</v>
       </c>
-      <c r="D31" s="7">
-        <v>640</v>
-      </c>
-      <c r="E31" s="7">
-        <v>610</v>
-      </c>
-      <c r="F31" s="7">
-        <v>560</v>
+      <c r="D31" s="6">
+        <f>'Cost Build'!D25</f>
+        <v>577.5</v>
+      </c>
+      <c r="E31" s="6">
+        <f>'Cost Build'!E25</f>
+        <v>511.5</v>
+      </c>
+      <c r="F31" s="6">
+        <f>'Cost Build'!F25</f>
+        <v>440</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -2091,15 +2229,15 @@
       </c>
       <c r="D32" s="9">
         <f>D30-D31</f>
-        <v>10510</v>
+        <v>10595.99</v>
       </c>
       <c r="E32" s="9">
         <f>E30-E31</f>
-        <v>12850</v>
+        <v>12456.056747499992</v>
       </c>
       <c r="F32" s="9">
         <f>F30-F31</f>
-        <v>16130</v>
+        <v>15191.025819582497</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -2108,15 +2246,15 @@
       </c>
       <c r="D33" s="9">
         <f>ROUND(D32*TaxRate,0)</f>
-        <v>2628</v>
+        <v>2649</v>
       </c>
       <c r="E33" s="9">
         <f>ROUND(E32*TaxRate,0)</f>
-        <v>3213</v>
+        <v>3114</v>
       </c>
       <c r="F33" s="9">
         <f>ROUND(F32*TaxRate,0)</f>
-        <v>4033</v>
+        <v>3798</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -2125,15 +2263,15 @@
       </c>
       <c r="D35" s="10">
         <f>D32-D33</f>
-        <v>7882</v>
+        <v>7946.99</v>
       </c>
       <c r="E35" s="10">
         <f>E32-E33</f>
-        <v>9637</v>
+        <v>9342.0567474999916</v>
       </c>
       <c r="F35" s="10">
         <f>F32-F33</f>
-        <v>12097</v>
+        <v>11393.025819582497</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
@@ -2142,35 +2280,736 @@
       </c>
       <c r="D36" s="13">
         <f>IF(D10=0,0,D35/D10)</f>
-        <v>0.16420833333333335</v>
+        <v>0.1655967909981246</v>
       </c>
       <c r="E36" s="13">
         <f>IF(E10=0,0,E35/E10)</f>
-        <v>0.17846296296296296</v>
+        <v>0.17313770943556314</v>
       </c>
       <c r="F36" s="13">
         <f>IF(F10=0,0,F35/F10)</f>
-        <v>0.19831147540983607</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C39" t="s">
-        <v>87</v>
-      </c>
-      <c r="D39" s="14">
-        <v>0.25</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>88</v>
+        <v>0.187517203750797</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="3" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="6" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" s="14">
+        <f>Assumptions!D8</f>
+        <v>95000</v>
+      </c>
+      <c r="E8" s="14">
+        <f>D8*(1+Assumptions!E9)</f>
+        <v>103550.00000000001</v>
+      </c>
+      <c r="F8" s="14">
+        <f>E8*(1+Assumptions!F9)</f>
+        <v>111834.00000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" s="15">
+        <f>Assumptions!D10</f>
+        <v>402</v>
+      </c>
+      <c r="E9" s="15">
+        <f>D9*(1+Assumptions!E11)</f>
+        <v>412.04999999999995</v>
+      </c>
+      <c r="F9" s="15">
+        <f>E9*(1+Assumptions!F11)</f>
+        <v>422.35124999999994</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="8">
+        <f>D8*D9/1000</f>
+        <v>38190</v>
+      </c>
+      <c r="E10" s="8">
+        <f>E8*E9/1000</f>
+        <v>42667.777499999997</v>
+      </c>
+      <c r="F10" s="8">
+        <f>F8*F9/1000</f>
+        <v>47233.229692500005</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13" s="16">
+        <f>Assumptions!D12</f>
+        <v>140</v>
+      </c>
+      <c r="E13" s="16">
+        <f>D13*(1+Assumptions!E13)</f>
+        <v>156.80000000000001</v>
+      </c>
+      <c r="F13" s="16">
+        <f>E13*(1+Assumptions!F13)</f>
+        <v>180.32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>92</v>
+      </c>
+      <c r="D14" s="16">
+        <f>Assumptions!D14</f>
+        <v>70</v>
+      </c>
+      <c r="E14" s="16">
+        <f>Assumptions!E14</f>
+        <v>72</v>
+      </c>
+      <c r="F14" s="16">
+        <f>Assumptions!F14</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="8">
+        <f>D13*D14</f>
+        <v>9800</v>
+      </c>
+      <c r="E15" s="8">
+        <f>E13*E14</f>
+        <v>11289.6</v>
+      </c>
+      <c r="F15" s="8">
+        <f>F13*F14</f>
+        <v>13524</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" s="10">
+        <f>D10+D15</f>
+        <v>47990</v>
+      </c>
+      <c r="E17" s="10">
+        <f>E10+E15</f>
+        <v>53957.377499999995</v>
+      </c>
+      <c r="F17" s="10">
+        <f>F10+F15</f>
+        <v>60757.229692500005</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="3" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="6" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" s="14">
+        <f>'Revenue Build'!D8</f>
+        <v>95000</v>
+      </c>
+      <c r="E8" s="14">
+        <f>'Revenue Build'!E8</f>
+        <v>103550.00000000001</v>
+      </c>
+      <c r="F8" s="14">
+        <f>'Revenue Build'!F8</f>
+        <v>111834.00000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="15">
+        <f>Assumptions!D17</f>
+        <v>181</v>
+      </c>
+      <c r="E9" s="15">
+        <f>D9*(1+Assumptions!E18)</f>
+        <v>186.43</v>
+      </c>
+      <c r="F9" s="15">
+        <f>E9*(1+Assumptions!F18)</f>
+        <v>192.02290000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="8">
+        <f>D8*D9/1000</f>
+        <v>17195</v>
+      </c>
+      <c r="E10" s="8">
+        <f>E8*E9/1000</f>
+        <v>19304.826500000003</v>
+      </c>
+      <c r="F10" s="8">
+        <f>F8*F9/1000</f>
+        <v>21474.688998600006</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="16">
+        <f>D8*Assumptions!D19/1000</f>
+        <v>76</v>
+      </c>
+      <c r="E12" s="16">
+        <f>E8*Assumptions!E19/1000</f>
+        <v>81.804500000000019</v>
+      </c>
+      <c r="F12" s="16">
+        <f>F8*Assumptions!F19/1000</f>
+        <v>87.230520000000013</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="17">
+        <f>D12*Assumptions!D20</f>
+        <v>7600</v>
+      </c>
+      <c r="E13" s="17">
+        <f>E12*Assumptions!E20</f>
+        <v>8507.6680000000015</v>
+      </c>
+      <c r="F13" s="17">
+        <f>F12*Assumptions!F20</f>
+        <v>9420.8961600000021</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>76</v>
+      </c>
+      <c r="D16" s="6">
+        <f>Assumptions!D23*Assumptions!D25</f>
+        <v>3900</v>
+      </c>
+      <c r="E16" s="6">
+        <f>Assumptions!E23*Assumptions!E25</f>
+        <v>4262.5</v>
+      </c>
+      <c r="F16" s="6">
+        <f>Assumptions!F23*Assumptions!F25</f>
+        <v>4582</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>79</v>
+      </c>
+      <c r="D17" s="6">
+        <f>Assumptions!D24*Assumptions!D26</f>
+        <v>2700</v>
+      </c>
+      <c r="E17" s="6">
+        <f>Assumptions!E24*Assumptions!E26</f>
+        <v>2883</v>
+      </c>
+      <c r="F17" s="6">
+        <f>Assumptions!F24*Assumptions!F26</f>
+        <v>3040</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" s="6">
+        <f>'Revenue Build'!D17*Assumptions!D29</f>
+        <v>2351.5100000000002</v>
+      </c>
+      <c r="E20" s="6">
+        <f>'Revenue Build'!E17*Assumptions!E29</f>
+        <v>2751.8262524999996</v>
+      </c>
+      <c r="F20" s="6">
+        <f>'Revenue Build'!F17*Assumptions!F29</f>
+        <v>3098.6187143175002</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C21" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" s="6">
+        <f>Assumptions!D30</f>
+        <v>1450</v>
+      </c>
+      <c r="E21" s="6">
+        <f>Assumptions!E30</f>
+        <v>1500</v>
+      </c>
+      <c r="F21" s="6">
+        <f>Assumptions!F30</f>
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C24" t="s">
+        <v>101</v>
+      </c>
+      <c r="D24" s="6">
+        <f>'Balance Sheet'!D26+'Balance Sheet'!D30</f>
+        <v>10500</v>
+      </c>
+      <c r="E24" s="6">
+        <f>'Balance Sheet'!E26+'Balance Sheet'!E30</f>
+        <v>9300</v>
+      </c>
+      <c r="F24" s="6">
+        <f>'Balance Sheet'!F26+'Balance Sheet'!F30</f>
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>82</v>
+      </c>
+      <c r="D25" s="17">
+        <f>D24*Assumptions!D31</f>
+        <v>577.5</v>
+      </c>
+      <c r="E25" s="17">
+        <f>E24*Assumptions!E31</f>
+        <v>511.5</v>
+      </c>
+      <c r="F25" s="17">
+        <f>F24*Assumptions!F31</f>
+        <v>440</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="3" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="6" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" s="18">
+        <v>95000</v>
+      </c>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19">
+        <v>0.09</v>
+      </c>
+      <c r="F9" s="19">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" s="18">
+        <v>402</v>
+      </c>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>108</v>
+      </c>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="F11" s="19">
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>109</v>
+      </c>
+      <c r="D12" s="18">
+        <v>140</v>
+      </c>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19">
+        <v>0.12</v>
+      </c>
+      <c r="F13" s="19">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D14" s="20">
+        <v>70</v>
+      </c>
+      <c r="E14" s="20">
+        <v>72</v>
+      </c>
+      <c r="F14" s="20">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>113</v>
+      </c>
+      <c r="D17" s="18">
+        <v>181</v>
+      </c>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C18" t="s">
+        <v>114</v>
+      </c>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19">
+        <v>0.03</v>
+      </c>
+      <c r="F18" s="19">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>115</v>
+      </c>
+      <c r="D19" s="21">
+        <v>0.8</v>
+      </c>
+      <c r="E19" s="21">
+        <v>0.79</v>
+      </c>
+      <c r="F19" s="21">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>116</v>
+      </c>
+      <c r="D20" s="18">
+        <v>100</v>
+      </c>
+      <c r="E20" s="18">
+        <v>104</v>
+      </c>
+      <c r="F20" s="18">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" s="18">
+        <v>52</v>
+      </c>
+      <c r="E23" s="18">
+        <v>55</v>
+      </c>
+      <c r="F23" s="18">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C24" t="s">
+        <v>119</v>
+      </c>
+      <c r="D24" s="18">
+        <v>30</v>
+      </c>
+      <c r="E24" s="18">
+        <v>31</v>
+      </c>
+      <c r="F24" s="18">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" s="20">
+        <v>75</v>
+      </c>
+      <c r="E25" s="20">
+        <v>77.5</v>
+      </c>
+      <c r="F25" s="20">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
+        <v>121</v>
+      </c>
+      <c r="D26" s="20">
+        <v>90</v>
+      </c>
+      <c r="E26" s="20">
+        <v>93</v>
+      </c>
+      <c r="F26" s="20">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C29" t="s">
+        <v>123</v>
+      </c>
+      <c r="D29" s="19">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="E29" s="19">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="F29" s="19">
+        <v>5.0999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C30" t="s">
+        <v>124</v>
+      </c>
+      <c r="D30" s="7">
+        <v>1450</v>
+      </c>
+      <c r="E30" s="7">
+        <v>1500</v>
+      </c>
+      <c r="F30" s="7">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C31" t="s">
+        <v>125</v>
+      </c>
+      <c r="D31" s="19">
+        <v>5.5E-2</v>
+      </c>
+      <c r="E31" s="19">
+        <v>5.5E-2</v>
+      </c>
+      <c r="F31" s="19">
+        <v>5.5E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C32" t="s">
+        <v>126</v>
+      </c>
+      <c r="D32" s="22">
+        <v>0.25</v>
+      </c>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>